<commit_message>
Footing excavation with fixed levels; F.B.L 1109.5 rafts deeper
Area 1 from 1114.85 to 1113.0, except the north-west 50 cm raft and the
west 80 cm raft (F.B.L 1109.5) taken from 1114.85 to 1109.5; area 2 from
1120.9 to 1118.0. Volumes over the blinding of footings and rafts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/footing_excavation.xlsx
+++ b/footing_excavation.xlsx
@@ -60,9 +60,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,18 +427,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,42 +447,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Blinding area (m²)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Bottom level</t>
-        </is>
-      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Bulk exc. level</t>
+          <t>From level</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>A) below bulk level (m³)</t>
+          <t>To level</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>B) from ground (m³)</t>
+          <t>Depth (m)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ground min</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Ground mean</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Ground max</t>
+          <t>Volume (m³)</t>
         </is>
       </c>
     </row>
@@ -496,237 +482,176 @@
           <t>Area 1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1629.83</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Footings &amp; rafts</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>1113</v>
+        <v>1433.56</v>
       </c>
       <c r="D2" t="n">
         <v>1114.85</v>
       </c>
       <c r="E2" t="n">
-        <v>2948.02</v>
+        <v>1113</v>
       </c>
       <c r="F2" t="n">
-        <v>9820.620000000001</v>
+        <v>1.85</v>
       </c>
       <c r="G2" t="n">
-        <v>1111.88</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1119.02</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1126.17</v>
+        <v>2652.09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Area 2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>258.98</v>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>North-west raft 50 cm (F.B.L 1109.5)</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>1118</v>
+        <v>77.23</v>
       </c>
       <c r="D3" t="n">
-        <v>1120.9</v>
+        <v>1114.85</v>
       </c>
       <c r="E3" t="n">
-        <v>751.04</v>
+        <v>1109.5</v>
       </c>
       <c r="F3" t="n">
-        <v>1412.53</v>
+        <v>5.35</v>
       </c>
       <c r="G3" t="n">
-        <v>1121.48</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1123.45</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1126.39</v>
+        <v>413.18</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL (areas 1 + 2)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>1888.81</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="n">
-        <v>3699.06</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>11233.16</v>
-      </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>West raft 80 cm (F.B.L 1109.5)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>135.44</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1109.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="G4" t="n">
+        <v>724.58</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Outside both hatched areas (not counted)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>23.79</v>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Footings &amp; rafts</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>266.37</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1118</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>772.48</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Of which inside hangar / rooms zones</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Blinding area (m²)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>A) (m³)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>B) (m³)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1646.23</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>3789.85</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Area 1 - inside hangar/rooms</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>483.13</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>266.37</v>
+      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="n">
-        <v>882.53</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1597.89</v>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>772.48</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Area 1 - outside hangar/rooms</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1146.7</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="n">
-        <v>2065.49</v>
-      </c>
-      <c r="F9" t="n">
-        <v>8222.74</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Area 2 - inside hangar/rooms</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>22.83</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="n">
-        <v>66.22</v>
-      </c>
-      <c r="F10" t="n">
-        <v>148.02</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="n">
+        <v>1912.6</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="n">
+        <v>4562.32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Area 2 - outside hangar/rooms</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>236.14</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>684.8200000000001</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1264.51</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
           <t>Footprint</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>blinding under footings &amp; rafts, ground beams excluded (FOUNDATIONS.dxf)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Ground</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>grid levels lowered by 0.25 m, bilinear inside each 3 m square</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>A)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>from min(ground, bulk excavation level) down to the bottom level</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>B)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>from ground level down to the bottom level</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Footing excavation: per-footing breakdown sheet and labels
Lists every isolated footing F1-F10 (16 No.) with its blinding
(A+0.2)x(B+0.2), the area it stands in, levels and volume; the rest of the
blinding is reported as rafts / tank / wall footings. Footings are numbered
on the drawing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/footing_excavation.xlsx
+++ b/footing_excavation.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Footing excavation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="By footing" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -58,10 +59,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -658,4 +662,948 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Footing</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>A x B (m)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Blinding (A+0.2)x(B+0.2) (m²)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Depth (m)</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Volume (m³)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Site X</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Site Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4.00 x 4.00</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I2" t="n">
+        <v>32.63</v>
+      </c>
+      <c r="J2" t="n">
+        <v>353770.55</v>
+      </c>
+      <c r="K2" t="n">
+        <v>355973.95</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3.80 x 3.80</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I3" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>353777.7</v>
+      </c>
+      <c r="K3" t="n">
+        <v>355973.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3.80 x 3.80</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I4" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="J4" t="n">
+        <v>353788.82</v>
+      </c>
+      <c r="K4" t="n">
+        <v>355971.77</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>8.75 x 5.00</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>46.54</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I5" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>353769.58</v>
+      </c>
+      <c r="K5" t="n">
+        <v>355965.79</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>9.35 x 6.00</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I6" t="n">
+        <v>109.54</v>
+      </c>
+      <c r="J6" t="n">
+        <v>353776.74</v>
+      </c>
+      <c r="K6" t="n">
+        <v>355965.03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>9.35 x 6.00</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I7" t="n">
+        <v>109.54</v>
+      </c>
+      <c r="J7" t="n">
+        <v>353787.86</v>
+      </c>
+      <c r="K7" t="n">
+        <v>355963.71</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5.10 x 5.10</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>28.09</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I8" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="J8" t="n">
+        <v>353768.26</v>
+      </c>
+      <c r="K8" t="n">
+        <v>355954.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>6.50 x 6.50</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>44.89</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I9" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="J9" t="n">
+        <v>353775.41</v>
+      </c>
+      <c r="K9" t="n">
+        <v>355953.94</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6.00 x 6.00</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>38.44</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I10" t="n">
+        <v>71.11</v>
+      </c>
+      <c r="J10" t="n">
+        <v>353786.54</v>
+      </c>
+      <c r="K10" t="n">
+        <v>355952.61</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5.10 x 5.10</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>28.09</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I11" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="J11" t="n">
+        <v>353767.19</v>
+      </c>
+      <c r="K11" t="n">
+        <v>355945.86</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>6.70 x 6.70</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>47.61</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I12" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="J12" t="n">
+        <v>353774.34</v>
+      </c>
+      <c r="K12" t="n">
+        <v>355945.01</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>6.50 x 6.50</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>44.89</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I13" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="J13" t="n">
+        <v>353785.46</v>
+      </c>
+      <c r="K13" t="n">
+        <v>355943.68</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3.60 x 3.60</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14.44</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1118</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I14" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="J14" t="n">
+        <v>353801.21</v>
+      </c>
+      <c r="K14" t="n">
+        <v>355929.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2.30 x 1.90</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I15" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="J15" t="n">
+        <v>353792.67</v>
+      </c>
+      <c r="K15" t="n">
+        <v>355927.25</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2.30 x 1.90</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1118</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I16" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="J16" t="n">
+        <v>353796.73</v>
+      </c>
+      <c r="K16" t="n">
+        <v>355926.76</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2.30 x 1.90</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1118</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I17" t="n">
+        <v>15.23</v>
+      </c>
+      <c r="J17" t="n">
+        <v>353800.92</v>
+      </c>
+      <c r="K17" t="n">
+        <v>355926.27</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Footings in area 1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>451.86</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>835.9400000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Footings in area 2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>24.94</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>72.33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ALL FOOTINGS (16)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="n">
+        <v>476.8</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="n">
+        <v>908.27</v>
+      </c>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Rafts, water tank and wall footings (rest of the blinding)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Area 1: rafts / tank / walls</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>981.7</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1113</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1816.15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Area 1: North-west raft 50 cm (F.B.L 1109.5)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>77.23</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1109.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I25" t="n">
+        <v>413.18</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Area 1: West raft 80 cm (F.B.L 1109.5)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>135.44</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Area 1</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1114.85</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1109.5</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I26" t="n">
+        <v>724.58</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Area 2: rafts / tank / walls</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>241.43</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Area 2</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1120.9</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1118</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I27" t="n">
+        <v>700.15</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL (footings + rafts)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="n">
+        <v>1912.6</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="n">
+        <v>4562.32</v>
+      </c>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>